<commit_message>
Add a reusable play-on screen, a coin wallet and a test rewarded ad
- IPlayOnLevel lets any mode's round be continued; FlagQuizRound implements it
- PlayOnSession applies the economy rules: coins restore all hearts or add 30 s, with prices rising per use;
  a rewarded video gives 1 heart or 10 s without raising the price
- PlayOnPanel: the "keep playing?" screen, reusable by every mode, wired into Flag Quizz
- Wallet with coins saved on the device; new players start with wallet.start_coins (new sheet key, 200)
- Clearing a level now pays reward.level_clear coins plus a bonus per star
- TestRewardedAds stands in for the ad network behind IRewardedAds

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FR8grRNJYREAYnkk1ZcrT3
</commit_message>
<xml_diff>
--- a/Tools/economy/economy_config.xlsx
+++ b/Tools/economy/economy_config.xlsx
@@ -457,9 +457,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -527,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2144,7 +2142,6 @@
           <t>bool</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
           <t>Ads</t>
@@ -2230,7 +2227,6 @@
           <t>bool</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
           <t>Ads</t>
@@ -2256,7 +2252,6 @@
           <t>bool</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
           <t>Ads</t>
@@ -2282,7 +2277,6 @@
           <t>bool</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
           <t>Ads</t>
@@ -2468,7 +2462,6 @@
           <t>Store (EUR)</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2524,7 +2517,6 @@
           <t>Store (EUR)</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2580,7 +2572,6 @@
           <t>Store (EUR)</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2636,12 +2627,41 @@
           <t>Store (EUR)</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>wallet.start_coins</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>coins</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Wallet</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Coins a new player starts with</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F71"/>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C2:C72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"int,float,bool,string"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2704,7 +2724,6 @@
       <c r="B3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2730,7 +2749,6 @@
       <c r="B5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2742,7 +2760,6 @@
         <f>B2*(Config!$B$42+B3*Config!$B$43)</f>
         <v/>
       </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2754,7 +2771,6 @@
         <f>B2/Config!$B$45*(Config!$B$46+Config!$B$47)/2</f>
         <v/>
       </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2766,7 +2782,6 @@
         <f>MIN(B4,Config!$B$53)*Config!$B$52</f>
         <v/>
       </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2778,7 +2793,6 @@
         <f>B5*(Config!$B$48+Config!$B$49)/2</f>
         <v/>
       </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2838,7 +2852,6 @@
         <f>Config!$B$65/Config!$B$64</f>
         <v/>
       </c>
-      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">

</xml_diff>

<commit_message>
Play-on, coins, lives and navigation (#4)
Reusable play-on screen with coins and a test rewarded ad, coin wallet and level rewards, lives with regen, Home with quit confirmation in Flag Quizz, and Back on other screens.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FR8grRNJYREAYnkk1ZcrT3
</commit_message>
<xml_diff>
--- a/Tools/economy/economy_config.xlsx
+++ b/Tools/economy/economy_config.xlsx
@@ -457,9 +457,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -527,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2144,7 +2142,6 @@
           <t>bool</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
           <t>Ads</t>
@@ -2230,7 +2227,6 @@
           <t>bool</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
           <t>Ads</t>
@@ -2256,7 +2252,6 @@
           <t>bool</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
           <t>Ads</t>
@@ -2282,7 +2277,6 @@
           <t>bool</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
           <t>Ads</t>
@@ -2468,7 +2462,6 @@
           <t>Store (EUR)</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2524,7 +2517,6 @@
           <t>Store (EUR)</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2580,7 +2572,6 @@
           <t>Store (EUR)</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2636,12 +2627,41 @@
           <t>Store (EUR)</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>wallet.start_coins</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>coins</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Wallet</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Coins a new player starts with</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F71"/>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C2:C72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"int,float,bool,string"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2704,7 +2724,6 @@
       <c r="B3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2730,7 +2749,6 @@
       <c r="B5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2742,7 +2760,6 @@
         <f>B2*(Config!$B$42+B3*Config!$B$43)</f>
         <v/>
       </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2754,7 +2771,6 @@
         <f>B2/Config!$B$45*(Config!$B$46+Config!$B$47)/2</f>
         <v/>
       </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2766,7 +2782,6 @@
         <f>MIN(B4,Config!$B$53)*Config!$B$52</f>
         <v/>
       </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2778,7 +2793,6 @@
         <f>B5*(Config!$B$48+Config!$B$49)/2</f>
         <v/>
       </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2838,7 +2852,6 @@
         <f>Config!$B$65/Config!$B$64</f>
         <v/>
       </c>
-      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">

</xml_diff>